<commit_message>
P00: cuenta 10 para todo el que hizo push, que era su objetivo
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -10,16 +10,10 @@
     <sheet name="Matriz" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="322098930" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="323290577" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="321094427" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="316087045" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="322179684" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="322330157" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="323298535" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="323065115" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="319112375" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="322153686" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="426058988" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="323272733" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="323298535" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="323065115" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="319112375" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -644,7 +638,7 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>La T01 vence el lunes 14-sep. El .class no se contabiliza en P00-P03: el repositorio lo estaba ignorando por error (ya corregido).</t>
+          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo al repositorio. La T01 vence el lunes 14-sep. El .class no se contabiliza: el repositorio lo estaba ignorando por error (ya corregido).</t>
         </is>
       </c>
     </row>
@@ -802,9 +796,9 @@
           <t>323072461</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C10" s="7" t="inlineStr">
@@ -1098,9 +1092,9 @@
           <t>321094427</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B18" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
@@ -1135,9 +1129,9 @@
           <t>316087045</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -1246,9 +1240,9 @@
           <t>322330157</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B22" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -1283,9 +1277,9 @@
           <t>426058256</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -1394,9 +1388,9 @@
           <t>319112375</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="B26" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
@@ -1579,9 +1573,9 @@
           <t>322153686</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -1616,9 +1610,9 @@
           <t>321337964</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="B32" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -1653,9 +1647,9 @@
           <t>426058988</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -1727,9 +1721,9 @@
           <t>323272733</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -1768,7 +1762,7 @@
     <row r="38">
       <c r="A38" s="14" t="inlineStr">
         <is>
-          <t>P00:  correctas 17   ·   pendientes de correccion 6   ·   no presentadas 6</t>
+          <t>P00:  correctas 27   ·   pendientes de correccion 0   ·   no presentadas 2</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1790,7 @@
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Las cuatro completas y correctas: 5 de 29     ·     Sin ninguna entrega: 2 de 29</t>
+          <t>Las cuatro completas y correctas: 7 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
@@ -1804,522 +1798,6 @@
       <c r="A43" s="16" t="inlineStr">
         <is>
           <t>T01 (vence el 14-sep): 1 entrega anticipada</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 319112375</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 319112375   ·   Por corregir: P03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: NP    P01: NP    P02: NP    P03: PC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas. Tu Laboratorio.java esta identico al que se te dio.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Descomentalas y completalas, y vuelve a subir el archivo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>No entregaste el documento con tu analisis, que es la mitad de la calificacion.</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Corre el programa, toma captura de la tabla final y escribe por que fallaste las 4 que fallaste. Acertaste 32 de 36: te falta poco.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 322153686</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 322153686   ·   Por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC    P01: 9    P02: 10    P03: NP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu P00 es un HolaMundo.java. La P00 pedia un archivo de texto con tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Crea un .txt en tu carpeta p00 con tu nombre completo adentro y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 426058988</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 426058988   ·   Por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC    P01: 10    P02: 10    P03: NP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu P00 sigue sin llevar tu nombre: dice 'Practica 00, creo que si es asi unu'.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Abre ese archivo, escribe tu nombre completo, guarda y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 323272733</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 323272733   ·   Por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC    P01: 10    P02: 10    P03: NP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu P00 dice 'Hola profe :) PRUEBA' pero no trae tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Abre ese archivo, escribe tu nombre completo y haz push.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
         </is>
       </c>
     </row>
@@ -2608,21 +2086,21 @@
     <row r="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
-          <t>Correccion · 321094427</t>
+          <t>Correccion · 322179684</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 321094427   ·   Por corregir: P00</t>
+          <t>Cuenta: 322179684   ·   Por corregir: P02</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: PC    P01: NP    P02: NP    P03: NP</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: NP</t>
         </is>
       </c>
     </row>
@@ -2641,12 +2119,12 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Tu P00 es un HolaMundo.java que imprime 'Hola, mundo'. La P00 pedia un archivo de TEXTO con tu nombre: era la prueba de que sabes hacer push.</t>
+          <t>Tu variante de constructores ya quedo: le agregamos el constructor que faltaba desde tu rama vieja y ya compila.</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Crea entregas/tu_apellido_nombre/p00/prueba.txt con tu nombre completo adentro y haz push. Guarda tu HolaMundo para la P01.</t>
+          <t>No tienes que hacer nada aqui. Solo trabaja de aqui en adelante en tu rama entregas_, no en las viejas.</t>
         </is>
       </c>
     </row>
@@ -2719,384 +2197,6 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 316087045</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 316087045   ·   Por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC    P01: 10    P02: NP    P03: NP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu p00 y tu p01 son el mismo archivo. La P00 pedia un archivo de TEXTO con tu nombre, no un programa.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Crea entregas/tu_apellido_nombre/p00/prueba.txt con tu nombre completo adentro. Tu P01 ya esta bien, esa dejala.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 322179684</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 322179684   ·   Por corregir: P02</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: NP</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu variante de constructores ya quedo: le agregamos el constructor que faltaba desde tu rama vieja y ya compila.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>No tienes que hacer nada aqui. Solo trabaja de aqui en adelante en tu rama entregas_, no en las viejas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
-          <t>Correccion · 322330157</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 322330157   ·   Por corregir: P00</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: PC    P01: 9    P02: 10    P03: 10</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Tu P00 es un HolaMundo.java, no un txt con tu nombre.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Crea entregas/tu_apellido_nombre/p00/prueba.txt con tu nombre completo adentro y haz push. Tu P03 quedo muy bien.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3246,7 +2346,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3382,4 +2482,142 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Correccion · 319112375</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 319112375   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: NP    P02: NP    P03: PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="18" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="19" t="inlineStr">
+        <is>
+          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas. Tu Laboratorio.java esta identico al que se te dio.</t>
+        </is>
+      </c>
+      <c r="B6" s="19" t="inlineStr">
+        <is>
+          <t>Descomentalas y completalas, y vuelve a subir el archivo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="19" t="inlineStr">
+        <is>
+          <t>No entregaste el documento con tu analisis, que es la mitad de la calificacion.</t>
+        </is>
+      </c>
+      <c r="B7" s="19" t="inlineStr">
+        <is>
+          <t>Corre el programa, toma captura de la tabla final y escribe por que fallaste las 4 que fallaste. Acertaste 32 de 36: te falta poco.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="21" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="21" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="21" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="21" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
P03: la corrida rapida para probar el bloque 7 no penaliza, y se documenta en la guia
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -1553,7 +1553,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F30" s="9" t="inlineStr">
@@ -1563,7 +1563,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>La mejor puntuacion del grupo (33/36) y tu documento esta completo. Detalle: el mis-resultados.txt que subiste es de una corrida de prueba y contradice tu documento.</t>
+          <t>La mejor puntuacion del grupo (33/36) y tu documento completo. Entrega correcta.</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2202,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B18"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2266,76 +2266,64 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="19" t="inlineStr">
-        <is>
-          <t>El mis-resultados.txt que subiste es de una corrida de prueba: contestaste '1' a las 36 y marca 1 DE 36.</t>
-        </is>
-      </c>
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>Sube el que corresponde a tu documento (25 de 36), o borralo: tu PDF ya trae la tabla buena.</t>
+    <row r="9">
+      <c r="A9" s="20" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A10" s="21" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>git fetch origin</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
+          <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="21" t="inlineStr">
         <is>
-          <t>git commit -m "PNN: correccion"</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>

<commit_message>
P03: se acepta en 10 el analisis que cumple aunque sea breve
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -11,9 +11,8 @@
     <sheet name="322098930" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="323290577" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="323298535" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="323065115" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="319112375" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="323065115" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="319112375" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1331,7 +1330,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F24" s="9" t="inlineStr">
@@ -1341,7 +1340,7 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>El mejor analisis del grupo. Pero tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre. Ver tu hoja.</t>
+          <t>El mejor analisis del grupo, aceptada. Para que lo tengas: tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre.</t>
         </is>
       </c>
     </row>
@@ -2202,7 +2201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -2212,21 +2211,21 @@
     <row r="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
-          <t>Correccion · 323298535</t>
+          <t>Correccion · 323065115</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cuenta: 323298535   ·   Por corregir: P03</t>
+          <t>Cuenta: 323065115   ·   Por corregir: P03 · solo te falta el bloque 7</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 9    P02: 9    P03: 9</t>
+          <t>P00: 10    P01: 10    P02: 9    P03: PC</t>
         </is>
       </c>
     </row>
@@ -2245,85 +2244,73 @@
     <row r="6" ht="45" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
         <is>
-          <t>Tu 7.2 imprime true y se pedia false. Escribiste 47 % 2 != 0, que pregunta si es IMPAR.</t>
+          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas, tal como venia el archivo.</t>
         </is>
       </c>
       <c r="B6" s="19" t="inlineStr">
         <is>
-          <t>Se pedia una expresion que diga si es PAR: 47 % 2 == 0 . Tu propia captura muestra el 7.2 = true.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>Tu documento no trae tu nombre en ninguna parte.</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Ponle una portada con tu nombre y el de tu companero.</t>
+          <t>Descomentalas y completalas. Cada una tiene que ser una operacion de verdad, con un comentario diciendo que operador usaste.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="20" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
+      <c r="A9" s="21" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="21" t="inlineStr">
         <is>
-          <t>git fetch origin</t>
+          <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="21" t="inlineStr">
         <is>
-          <t>git checkout TU-RAMA</t>
+          <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="21" t="inlineStr">
         <is>
-          <t>git pull origin main</t>
+          <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="21" t="inlineStr">
         <is>
-          <t>(corrige tus archivos)</t>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="21" t="inlineStr">
         <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
+          <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="21" t="inlineStr">
         <is>
-          <t>git commit -m "PNN: correccion"</t>
+          <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2350,144 +2337,6 @@
     <row r="1">
       <c r="A1" s="17" t="inlineStr">
         <is>
-          <t>Correccion · 323065115</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Cuenta: 323065115   ·   Por corregir: P03</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: 10    P01: 10    P02: 9    P03: PC</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Que hay que corregir</t>
-        </is>
-      </c>
-      <c r="B5" s="18" t="inlineStr">
-        <is>
-          <t>Como se corrige</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
-        <is>
-          <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas, tal como venia el archivo.</t>
-        </is>
-      </c>
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>Descomentalas y completalas. Cada una tiene que ser una operacion de verdad, con un comentario diciendo que operador usaste.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
-        <is>
-          <t>Varias explicaciones de tu analisis son muy flojas ('no supimos que mas responder').</t>
-        </is>
-      </c>
-      <c r="B7" s="19" t="inlineStr">
-        <is>
-          <t>Lo que se califica es justo esa explicacion. Vuelve a esas y escribe que creias tu y que hace en realidad Java.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="20" t="inlineStr">
-        <is>
-          <t>Como subir la correccion</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="21" t="inlineStr">
-        <is>
-          <t>git fetch origin</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="21" t="inlineStr">
-        <is>
-          <t>git checkout TU-RAMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="21" t="inlineStr">
-        <is>
-          <t>git pull origin main</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="21" t="inlineStr">
-        <is>
-          <t>(corrige tus archivos)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="21" t="inlineStr">
-        <is>
-          <t>git add entregas/tu_apellido_nombre/pNN</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="21" t="inlineStr">
-        <is>
-          <t>git commit -m "PNN: correccion"</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="21" t="inlineStr">
-        <is>
-          <t>git push</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="22" t="inlineStr">
-        <is>
-          <t>No abras pull request: el push ES la entrega.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="62" customWidth="1" min="1" max="1"/>
-    <col width="78" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="17" t="inlineStr">
-        <is>
           <t>Correccion · 319112375</t>
         </is>
       </c>

</xml_diff>

<commit_message>
P03: 9 para quienes cumplieron todo salvo el bloque 7
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -884,9 +884,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="E12" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="F12" s="9" t="inlineStr">
@@ -896,7 +896,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>Tu P02 quedo corregida. En la P03 tu documento esta bien, pero no entregaste el Laboratorio.java del curso: subiste otro programa con los resultados escritos a mano y sin bloque 7. Ver tu hoja.</t>
+          <t>Tu P02 quedo corregida. Tu P03 se acepta en 9: tu documento esta bien, pero no entregaste el Laboratorio.java del curso ni el bloque 7. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1365,9 +1365,9 @@
           <t>9</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="E25" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="F25" s="9" t="inlineStr">
@@ -1377,7 +1377,7 @@
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>Tu documento esta completo, pero te falta escribir el bloque 7: sigue tal como venia. Ver tu hoja.</t>
+          <t>Aceptada en 9. Tu documento esta completo; lo unico que falto fue escribir el bloque 7: sigue tal como venia.</t>
         </is>
       </c>
     </row>
@@ -1782,14 +1782,14 @@
     <row r="41">
       <c r="A41" s="14" t="inlineStr">
         <is>
-          <t>P03:  correctas 7   ·   pendientes de correccion 3   ·   no presentadas 19</t>
+          <t>P03:  correctas 9   ·   pendientes de correccion 1   ·   no presentadas 19</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>Las cuatro completas y correctas: 7 de 29     ·     Sin ninguna entrega: 2 de 29</t>
+          <t>Las cuatro completas y correctas: 9 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
@@ -1835,7 +1835,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
         </is>
       </c>
     </row>
@@ -2225,7 +2225,7 @@
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 9    P03: PC</t>
+          <t>P00: 10    P01: 10    P02: 9    P03: 9</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte MPOO: T01 calificada y P03 cerrada sin pendientes
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="20">
+  <fonts count="19">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,12 +82,6 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="005B21B6"/>
-      <sz val="8"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
       <color rgb="00B45309"/>
       <sz val="10"/>
     </font>
@@ -138,7 +132,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -153,11 +147,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FEE2E2"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EDE9FE"/>
       </patternFill>
     </fill>
     <fill>
@@ -192,7 +181,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -219,23 +208,20 @@
     <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -630,14 +616,14 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>10 = correcta  ·  9 = correcta con un detalle de forma  ·  PC = pendiente de correccion (tienes hoja aparte)  ·  NP = no presentada  ·  — = aun no vence</t>
+          <t>10 = correcta  ·  9 = correcta con un detalle  ·  8 = incompleta pero aceptada  ·  PC = pendiente de correccion (tienes hoja aparte)  ·  NP = no presentada  ·  — = aun no vence</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo al repositorio. La T01 vence el lunes 14-sep. El .class no se contabiliza: el repositorio lo estaba ignorando por error (ya corregido).</t>
+          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo. T01: vence el lunes 14-sep, el guion (—) quiere decir que todavia no vence. El .class no se contabiliza: el repositorio lo estaba ignorando por error (ya corregido).</t>
         </is>
       </c>
     </row>
@@ -778,14 +764,14 @@
           <t>9</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>ENTREGADA</t>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Bloque 7 completo y buen analisis. Tu captura no muestra la tabla final, solo el final del reporte. Tu T01 ya llego y esta muy completa.</t>
+          <t>Bloque 7 completo y buen analisis; tu captura no muestra la tabla final, solo el final del reporte. Tu T01 esta muy bien: 10. Dos detalles para la proxima: a Television le falto la linea QUE IGNORE, y entre las tres clases no usaste la resta.</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1013,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>PC</t>
         </is>
@@ -1402,9 +1388,9 @@
           <t>NP</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
-        <is>
-          <t>PC</t>
+      <c r="E26" s="7" t="inlineStr">
+        <is>
+          <t>8</t>
         </is>
       </c>
       <c r="F26" s="9" t="inlineStr">
@@ -1414,7 +1400,7 @@
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>Contestaste las 36 y acertaste 32, de las mejores. Pero te falta todo el bloque 7 y el documento con tu analisis. Ver tu hoja.</t>
+          <t>Aceptada en 8. Contestaste las 36 y acertaste 32, de las mejores del grupo. Te falto el bloque 7 y el documento con tu analisis. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1752,51 +1738,51 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Resumen del grupo (29 alumnos)</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="14" t="inlineStr">
+      <c r="A38" s="13" t="inlineStr">
         <is>
           <t>P00:  correctas 27   ·   pendientes de correccion 0   ·   no presentadas 2</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="14" t="inlineStr">
+      <c r="A39" s="13" t="inlineStr">
         <is>
           <t>P01:  correctas 25   ·   pendientes de correccion 0   ·   no presentadas 4</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="14" t="inlineStr">
+      <c r="A40" s="13" t="inlineStr">
         <is>
           <t>P02:  correctas 21   ·   pendientes de correccion 1   ·   no presentadas 7</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="14" t="inlineStr">
-        <is>
-          <t>P03:  correctas 9   ·   pendientes de correccion 1   ·   no presentadas 19</t>
+      <c r="A41" s="13" t="inlineStr">
+        <is>
+          <t>P03:  correctas 10   ·   pendientes de correccion 0   ·   no presentadas 19</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="15" t="inlineStr">
+      <c r="A42" s="14" t="inlineStr">
         <is>
           <t>Las cuatro completas y correctas: 9 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="16" t="inlineStr">
-        <is>
-          <t>T01 (vence el 14-sep): 1 entrega anticipada</t>
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>T01 (vence el lunes 14-sep): 1 entrega anticipada, calificada</t>
         </is>
       </c>
     </row>
@@ -1819,7 +1805,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 322098930</t>
         </is>
@@ -1833,106 +1819,106 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>No entregaste el Laboratorio.java del curso. Subiste un programa propio que tiene los 36 resultados escritos a mano en un arreglo: no calcula nada, solo los imprime.</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, correlo, contesta las 36 y sube ESE archivo con tu bloque 7 escrito.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>Por lo mismo, no tienes bloque 7.</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Son las 5 lineas del final: descomentalas y completalas. Tu documento y tu analisis si estan bien, esos no le muevas.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -1957,7 +1943,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 323290577</t>
         </is>
@@ -1971,94 +1957,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: PC    P03: NP</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu P02 no compila: PruebaPunto3 y PruebaPunto4 crean el objeto con new Punto(5,8), pero tu clase Punto no tiene constructor con parametros.</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>O le agregas a Punto el constructor Punto(int x, int y), o cambias esas pruebas para que usen la clase que si lo tiene.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2083,7 +2069,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 322179684</t>
         </is>
@@ -2097,94 +2083,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: NP</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Tu variante de constructores ya quedo: le agregamos el constructor que faltaba desde tu rama vieja y ya compila.</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>No tienes que hacer nada aqui. Solo trabaja de aqui en adelante en tu rama entregas_, no en las viejas.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2209,7 +2195,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 323065115</t>
         </is>
@@ -2223,94 +2209,94 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="13" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 9    P03: 9</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas, tal como venia el archivo.</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Descomentalas y completalas. Cada una tiene que ser una operacion de verdad, con un comentario diciendo que operador usaste.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>
@@ -2335,7 +2321,7 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="17" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Correccion · 319112375</t>
         </is>
@@ -2349,106 +2335,106 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
-        <is>
-          <t>P00: 10    P01: NP    P02: NP    P03: PC</t>
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: NP    P02: NP    P03: 8</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B5" s="18" t="inlineStr">
+      <c r="B5" s="17" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="19" t="inlineStr">
+      <c r="A6" s="18" t="inlineStr">
         <is>
           <t>Te falta todo el bloque 7: las cinco lineas siguen comentadas. Tu Laboratorio.java esta identico al que se te dio.</t>
         </is>
       </c>
-      <c r="B6" s="19" t="inlineStr">
+      <c r="B6" s="18" t="inlineStr">
         <is>
           <t>Descomentalas y completalas, y vuelve a subir el archivo.</t>
         </is>
       </c>
     </row>
     <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="18" t="inlineStr">
         <is>
           <t>No entregaste el documento con tu analisis, que es la mitad de la calificacion.</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="18" t="inlineStr">
         <is>
           <t>Corre el programa, toma captura de la tabla final y escribe por que fallaste las 4 que fallaste. Acertaste 32 de 36: te falta poco.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="inlineStr">
+      <c r="A9" s="19" t="inlineStr">
         <is>
           <t>Como subir la correccion</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>git fetch origin</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>git checkout TU-RAMA</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>git pull origin main</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>(corrige tus archivos)</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>git add entregas/tu_apellido_nombre/pNN</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>git commit -m "PNN: correccion"</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>git push</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>No abras pull request: el push ES la entrega.</t>
         </is>

</xml_diff>

<commit_message>
Corte MPOO: limpia observaciones que ya no aplican
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -808,7 +808,7 @@
       </c>
       <c r="G10" s="10" t="inlineStr">
         <is>
-          <t>Faltan P00, P02 y P03.</t>
+          <t>Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
@@ -1104,7 +1104,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>Ya llego tu primera entrega. Tu P00 deberia ser un archivo de texto con tu nombre, no un HolaMundo.java. Ver tu hoja.</t>
+          <t>Ya llego tu primera entrega. Faltan la P01, la P02 y la P03.</t>
         </is>
       </c>
     </row>
@@ -1141,7 +1141,7 @@
       </c>
       <c r="G19" s="10" t="inlineStr">
         <is>
-          <t>Ya llego tu entrega y tu P01 esta bien. Tu P00 es el mismo archivo que la P01: deberia ser un .txt con tu nombre. Ver tu hoja.</t>
+          <t>Ya llego tu entrega y tu P01 esta bien. Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
@@ -1252,7 +1252,7 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'. Sigue pendiente tu P00.</t>
+          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
         </is>
       </c>
     </row>
@@ -1289,7 +1289,7 @@
       </c>
       <c r="G23" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 es la mas limpia del grupo, y entregaste tambien tu .class. Sigue pendiente tu P00.</t>
+          <t>Tu P03 es la mas limpia del grupo, y entregaste tambien tu .class.</t>
         </is>
       </c>
     </row>
@@ -1548,7 +1548,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>La mejor puntuacion del grupo (33/36) y tu documento completo. Entrega correcta.</t>
+          <t>Entrega correcta y completa.</t>
         </is>
       </c>
     </row>
@@ -1585,7 +1585,7 @@
       </c>
       <c r="G31" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero. Tu P00 sigue pendiente de corregir.</t>
+          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
         </is>
       </c>
     </row>
@@ -1622,7 +1622,7 @@
       </c>
       <c r="G32" s="10" t="inlineStr">
         <is>
-          <t>Tu P01 y P02 SI llegaron: estaban en dos ramas viejas y ya las pasamos a tu rama del semestre. Tu P01 no lleva tu nombre. Faltan la P00 y la P03.</t>
+          <t>Tu P01 y P02 SI llegaron: estaban en dos ramas viejas y ya las pasamos a tu rama del semestre. Tu P01 no lleva tu nombre. Falta la P03.</t>
         </is>
       </c>
     </row>
@@ -1659,7 +1659,7 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Tu P00 sigue sin llevar tu nombre adentro. Falta la P03. Ver tu hoja.</t>
+          <t>Falta la P03.</t>
         </is>
       </c>
     </row>
@@ -1696,7 +1696,7 @@
       </c>
       <c r="G34" s="10" t="inlineStr">
         <is>
-          <t>Tu P00 ya llego y con eso completas hasta la P02. Falta la P03.</t>
+          <t>Completa hasta la P02. Falta la P03.</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero. Tu P00 sigue pendiente.</t>
+          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte MPOO al 12-sep: cinco P03 que faltaban por revisar
</commit_message>
<xml_diff>
--- a/calificaciones/P00-P03-corte-11sep.xlsx
+++ b/calificaciones/P00-P03-corte-11sep.xlsx
@@ -13,6 +13,9 @@
     <sheet name="322179684" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="323065115" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="319112375" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="322287123" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="426058988" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="323272733" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -981,9 +984,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F15" s="9" t="inlineStr">
@@ -993,7 +996,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>Completa hasta P02. Falta la P03.</t>
+          <t>Completa. Detalle: en el bloque 7 no dejaste el comentario diciendo que operador usaste.</t>
         </is>
       </c>
     </row>
@@ -1166,9 +1169,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E20" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E20" s="7" t="inlineStr">
+        <is>
+          <t>10</t>
         </is>
       </c>
       <c r="F20" s="9" t="inlineStr">
@@ -1178,7 +1181,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>Tu P02 quedo corregida y ya compila. Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
+          <t>Completa. Dos detalles: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par', y tu explicacion del casting en (double) 7 / 2 no es correcta: no redondea, cambia el tipo de la division.</t>
         </is>
       </c>
     </row>
@@ -1425,9 +1428,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E27" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E27" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="F27" s="9" t="inlineStr">
@@ -1437,7 +1440,7 @@
       </c>
       <c r="G27" s="10" t="inlineStr">
         <is>
-          <t>Completa hasta P02. Falta la P03.</t>
+          <t>Tu bloque 7 esta completo y eres el unico que puso el comentario del operador en cada linea. Falto la captura de la TABLA FINAL, que era lo que se pedia, y tu analisis va por temas en vez de falla por falla.</t>
         </is>
       </c>
     </row>
@@ -1647,9 +1650,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E33" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>PC</t>
         </is>
       </c>
       <c r="F33" s="9" t="inlineStr">
@@ -1659,7 +1662,7 @@
       </c>
       <c r="G33" s="10" t="inlineStr">
         <is>
-          <t>Falta la P03.</t>
+          <t>Solo subiste el Laboratorio.class: falta el Laboratorio.java y el documento con tu captura y tu analisis, que es la mayor parte de la practica. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1721,9 +1724,9 @@
           <t>10</t>
         </is>
       </c>
-      <c r="E35" s="8" t="inlineStr">
-        <is>
-          <t>NP</t>
+      <c r="E35" s="7" t="inlineStr">
+        <is>
+          <t>9</t>
         </is>
       </c>
       <c r="F35" s="9" t="inlineStr">
@@ -1733,7 +1736,7 @@
       </c>
       <c r="G35" s="10" t="inlineStr">
         <is>
-          <t>Tu P03 no esta subida en tu rama, aunque apareces como equipo en el documento de tu companero.</t>
+          <t>Tu analisis es el mejor del grupo, muy bien. Pero no entregaste el Laboratorio.java de la practica: subiste otro programa con los resultados escritos a mano y sin el bloque 7. Ver tu hoja.</t>
         </is>
       </c>
     </row>
@@ -1768,14 +1771,14 @@
     <row r="41">
       <c r="A41" s="13" t="inlineStr">
         <is>
-          <t>P03:  correctas 10   ·   pendientes de correccion 0   ·   no presentadas 19</t>
+          <t>P03:  correctas 14   ·   pendientes de correccion 1   ·   no presentadas 14</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="14" t="inlineStr">
         <is>
-          <t>Las cuatro completas y correctas: 9 de 29     ·     Sin ninguna entrega: 2 de 29</t>
+          <t>Las cuatro completas y correctas: 13 de 29     ·     Sin ninguna entrega: 2 de 29</t>
         </is>
       </c>
     </row>
@@ -2085,7 +2088,7 @@
     <row r="3">
       <c r="A3" s="13" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 10    P02: 10    P03: NP</t>
+          <t>P00: 10    P01: 10    P02: 10    P03: 10</t>
         </is>
       </c>
     </row>
@@ -2443,4 +2446,418 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 322287123</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 322287123   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Falta la captura de la TABLA FINAL, la que dice 'TU TABLA FINAL · ESTA ES LA CAPTURA QUE TIENES QUE ENTREGAR'. Tu PDF termina en el bloque 6.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Corre el programa hasta el final y toma captura de esa tabla; tambien quedo guardada en mis-resultados.txt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Tu analisis va por temas y fallaste 13 predicciones.</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Lo que se califica es explicar CADA falla: que creias tu y que hace en realidad Java. Tu bloque 7 quedo muy bien, ese no le muevas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 426058988</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 426058988   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: PC</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="56" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>Solo subiste el Laboratorio.class. Falta el Laboratorio.java con tu bloque 7 y falta el documento con la captura de tu tabla final y tu analisis, que juntos son la mayor parte de la calificacion.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Sube tu Laboratorio.java y tu documento. Si ya corriste el programa, la tabla final tambien quedo en mis-resultados.txt, en la misma carpeta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Tu profesor va a revisar contigo esta entrega antes de calificarla.</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Acercate con el en la proxima sesion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="78" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="16" t="inlineStr">
+        <is>
+          <t>Correccion · 323272733</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Cuenta: 323272733   ·   Por corregir: P03</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="13" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 10    P02: 10    P03: 9</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="17" t="inlineStr">
+        <is>
+          <t>Que hay que corregir</t>
+        </is>
+      </c>
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>Como se corrige</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="18" t="inlineStr">
+        <is>
+          <t>No entregaste el Laboratorio.java de la practica: subiste un programa distinto, con los 36 resultados escritos a mano en un arreglo, que no calcula nada.</t>
+        </is>
+      </c>
+      <c r="B6" s="18" t="inlineStr">
+        <is>
+          <t>Baja el Laboratorio.java de guias-laboratorios/Lab-03/, escribe ahi tu bloque 7 y sube ESE archivo. Tu documento y tu analisis estan muy bien, esos no le muevas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="18" t="inlineStr">
+        <is>
+          <t>Por lo mismo, tu bloque 7 no existe (0 de 5).</t>
+        </is>
+      </c>
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>Son las cinco lineas del final: descomentalas y completalas con operaciones de verdad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="19" t="inlineStr">
+        <is>
+          <t>Como subir la correccion</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="20" t="inlineStr">
+        <is>
+          <t>git fetch origin</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="20" t="inlineStr">
+        <is>
+          <t>git checkout TU-RAMA</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="20" t="inlineStr">
+        <is>
+          <t>git pull origin main</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="20" t="inlineStr">
+        <is>
+          <t>(corrige tus archivos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="20" t="inlineStr">
+        <is>
+          <t>git add entregas/tu_apellido_nombre/pNN</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="20" t="inlineStr">
+        <is>
+          <t>git commit -m "PNN: correccion"</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="20" t="inlineStr">
+        <is>
+          <t>git push</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="21" t="inlineStr">
+        <is>
+          <t>No abras pull request: el push ES la entrega.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>